<commit_message>
ubah logika pencarian service fee
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/act/requirements_act.xlsx
+++ b/src/scrapers/output_scrape/act/requirements_act.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$300 (overseas), $300 (canberra)</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$300 (overseas), $300 (canberra)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
merevisi requirements.txt dan readme
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/act/requirements_act.xlsx
+++ b/src/scrapers/output_scrape/act/requirements_act.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -428,49 +443,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>state code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>state stream</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>General Requirements</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Requirements Canberra Residents</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Requirements overseas</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>service fee</t>
         </is>
       </c>
     </row>
     <row r="2" ht="409" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>ACT</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>190</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>The Skilled Nominated Visa (subclass 190) lets you live and work in Australia as a permanent resident. You must be nominated by a State or Territory government. Nomination triggers the visa invitation from the Department of Home Affairs.
 Two year commitment - If you are nominated by the ACT to apply for a 190 visa, you must live and work in Canberra for at least two years from visa grant, or if you are moving from overseas, date of arrival in Canberra.
@@ -486,7 +501,7 @@
 Overseas applicant eligibility</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -508,7 +523,7 @@
 Service fee : $300</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -534,24 +549,24 @@
 Service Fee : $300 Your supporting documentation must evidence your eligibility to apply for ACT nomination and any Matrix score claimed. Please refer to the key document checklist for more information on what documents you need to include.</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>$300 (overseas), $300 (canberra)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="409" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ACT</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>491</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>The Skilled Regional Work Visa (subclass 491) is a five year provisional visa for skilled workers to live and work in regional Australia. You must be nominated by a state or territory government. Nomination triggers the visa invitation from the Department of Home Affairs.
 Two year commitment - If you are nominated by the ACT to apply for a 491 visa, you must live and work in Canberra for at least two years from visa grant, or if you are moving from overseas, date of arrival in Canberra.
@@ -567,7 +582,7 @@
 Overseas applicant eligibility</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -587,7 +602,7 @@
 Service fee : $300</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -612,7 +627,7 @@
 Service Fee : $300</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>$300 (overseas), $300 (canberra)</t>
         </is>

</xml_diff>